<commit_message>
Patient Information: line-height fixes + importer aligned with the authored document (#375)
* cards brochure and columns related-links Line heigh fix

Automated migration updates generated by Experience Modernization Agent.

Changed files: 3

* Update importer

Automated migration updates generated by Experience Modernization Agent.

Changed files: 4

* Update importer

Automated migration updates generated by Experience Modernization Agent.

Changed files: 4

* Update 1 file

Automated migration updates generated by Experience Modernization Agent.

Changed files: 1

* Update 1 file

Automated migration updates generated by Experience Modernization Agent.

Changed files: 1

---------

Co-authored-by: AEMY Studio <noreply@aemy.studio>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-patient-information.report.xlsx
+++ b/tools/importer/reports/import-patient-information.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="120">
   <si>
     <t>_reportFile</t>
   </si>
@@ -70,6 +70,27 @@
     <t>https://patients.stryker.com/ww/en/stroke-awareness/resources.html</t>
   </si>
   <si>
+    <t>us/en/ent/search.report.json</t>
+  </si>
+  <si>
+    <t>["search"]</t>
+  </si>
+  <si>
+    <t>us/en/ent/search</t>
+  </si>
+  <si>
+    <t>search</t>
+  </si>
+  <si>
+    <t>2026-10-12T12:02:07.998Z</t>
+  </si>
+  <si>
+    <t>Search | Stryker</t>
+  </si>
+  <si>
+    <t>https://patients.stryker.com/us/en/ent/search.html</t>
+  </si>
+  <si>
     <t>us/en/ivs/get-the-facts.report.json</t>
   </si>
   <si>
@@ -79,10 +100,10 @@
     <t>us/en/ivs/get-the-facts</t>
   </si>
   <si>
-    <t>ivs-treatment</t>
-  </si>
-  <si>
-    <t>2026-09-28T14:16:18.644Z</t>
+    <t>ivs-get-the-facts</t>
+  </si>
+  <si>
+    <t>2026-10-12T10:30:18.552Z</t>
   </si>
   <si>
     <t>Get the facts | Stryker</t>
@@ -91,6 +112,27 @@
     <t>https://patients.stryker.com/us/en/ivs/get-the-facts.html</t>
   </si>
   <si>
+    <t>us/en/ivs/index.report.json</t>
+  </si>
+  <si>
+    <t>["hero","sticky-nav","columns","columns","columns","panel-gold","cards","statistics","statistics","panel-cta","panel-cta","panel-gold-cta","tabs"]</t>
+  </si>
+  <si>
+    <t>us/en/ivs/index</t>
+  </si>
+  <si>
+    <t>ivs-home</t>
+  </si>
+  <si>
+    <t>2026-09-28T18:00:39.028Z</t>
+  </si>
+  <si>
+    <t>Homepage | Stryker</t>
+  </si>
+  <si>
+    <t>https://patients.stryker.com/us/en/ivs/index.html</t>
+  </si>
+  <si>
     <t>us/en/stroke-awareness/patient-information.report.json</t>
   </si>
   <si>
@@ -103,7 +145,7 @@
     <t>patient-information</t>
   </si>
   <si>
-    <t>2026-10-02T09:42:22.620Z</t>
+    <t>2026-10-15T12:55:47.074Z</t>
   </si>
   <si>
     <t>Neurovascular Patient Information | Stryker</t>
@@ -248,6 +290,9 @@
   </si>
   <si>
     <t>us/en/ivs/treatments/mild</t>
+  </si>
+  <si>
+    <t>ivs-treatment</t>
   </si>
   <si>
     <t>2026-09-28T14:16:34.246Z</t>
@@ -720,7 +765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -886,47 +931,47 @@
         <v>38</v>
       </c>
       <c r="J5" t="s">
-        <v>18</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
         <v>42</v>
       </c>
       <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
         <v>43</v>
-      </c>
-      <c r="G6" t="s">
-        <v>12</v>
       </c>
       <c r="H6" t="s">
         <v>44</v>
       </c>
       <c r="I6" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="J6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -935,126 +980,126 @@
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
         <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J7" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="E8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="G8" t="s">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="H8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I8" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="J8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" t="s">
         <v>59</v>
-      </c>
-      <c r="B9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>49</v>
-      </c>
-      <c r="H9" t="s">
-        <v>61</v>
-      </c>
-      <c r="I9" t="s">
-        <v>62</v>
-      </c>
-      <c r="J9" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F10" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="G10" t="s">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="H10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I10" t="s">
-        <v>12</v>
+        <v>71</v>
       </c>
       <c r="J10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
@@ -1063,62 +1108,62 @@
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F11" t="s">
         <v>14</v>
       </c>
       <c r="G11" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="H11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="J11" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="E12" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F12" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="G12" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="H12" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="I12" t="s">
-        <v>78</v>
+        <v>12</v>
       </c>
       <c r="J12" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C13" t="s">
         <v>12</v>
@@ -1127,62 +1172,62 @@
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="H13" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="I13" t="s">
+        <v>87</v>
+      </c>
+      <c r="J13" t="s">
         <v>83</v>
-      </c>
-      <c r="J13" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>89</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F14" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>12</v>
+        <v>91</v>
       </c>
       <c r="H14" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I14" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="J14" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
@@ -1191,62 +1236,62 @@
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F15" t="s">
         <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="H15" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="I15" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="J15" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
       <c r="D16" t="s">
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="E16" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F16" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="G16" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="H16" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I16" t="s">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="J16" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C17" t="s">
         <v>12</v>
@@ -1255,22 +1300,86 @@
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F17" t="s">
         <v>14</v>
       </c>
       <c r="G17" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="H17" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="I17" t="s">
+        <v>108</v>
+      </c>
+      <c r="J17" t="s">
         <v>103</v>
       </c>
-      <c r="J17" t="s">
-        <v>104</v>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>110</v>
+      </c>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>63</v>
+      </c>
+      <c r="H18" t="s">
+        <v>111</v>
+      </c>
+      <c r="I18" t="s">
+        <v>112</v>
+      </c>
+      <c r="J18" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>116</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>63</v>
+      </c>
+      <c r="H19" t="s">
+        <v>117</v>
+      </c>
+      <c r="I19" t="s">
+        <v>118</v>
+      </c>
+      <c r="J19" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>